<commit_message>
feat: Reorganize batch 24 files and setup guides into a new 'daily' subdirectory, update one file, and remove unused assets.
</commit_message>
<xml_diff>
--- a/batches/24/day_27_28_29.xlsx
+++ b/batches/24/day_27_28_29.xlsx
@@ -8,13 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/ALI_2/work/acciojob/modules/sql/batches/24/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4AF83973-F573-C144-84F4-C93EDACB509F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5E3FBA3-FBAD-CC40-88E8-78A691DA1FB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29400" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="1" xr2:uid="{EAC50407-EEAA-A342-9C45-5B655C4B9469}"/>
+    <workbookView xWindow="29400" yWindow="0" windowWidth="38400" windowHeight="21600" activeTab="3" xr2:uid="{EAC50407-EEAA-A342-9C45-5B655C4B9469}"/>
   </bookViews>
   <sheets>
     <sheet name="Recap" sheetId="1" r:id="rId1"/>
     <sheet name="Agenda" sheetId="2" r:id="rId2"/>
+    <sheet name="Overview" sheetId="3" r:id="rId3"/>
+    <sheet name="Folder_Structure" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -87,6 +89,598 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>25776</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B7230C7-4E4C-1D8D-39E5-5F85DD5F069C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="203200"/>
+          <a:ext cx="7772400" cy="4496176"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>7861</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{373923DE-1A71-FBEE-2713-25E6BC569EB4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="4876800"/>
+          <a:ext cx="7772400" cy="6713461"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>58</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>91</xdr:row>
+      <xdr:rowOff>174885</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B02D52E0-09B7-10E9-49E9-A48AA1A4DA61}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="11785600"/>
+          <a:ext cx="7772400" cy="6880485"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>93</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>125</xdr:row>
+      <xdr:rowOff>124816</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{622B0218-D1DB-E8C9-C155-A4924BEED775}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="18897600"/>
+          <a:ext cx="7772400" cy="6627216"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>126</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>154</xdr:row>
+      <xdr:rowOff>22765</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="6" name="Picture 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1A4064CD-7FC7-E79F-5386-7A9E43E33B9F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="25603200"/>
+          <a:ext cx="7772400" cy="5712365"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>155</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>168</xdr:row>
+      <xdr:rowOff>77398</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93FCF794-4933-0297-48A8-02D535663127}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="31496000"/>
+          <a:ext cx="7772400" cy="2718998"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>44</xdr:row>
+      <xdr:rowOff>29156</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D1D2FF28-28B0-22E0-00B2-1F85B7D5E9CA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="203200"/>
+          <a:ext cx="7772400" cy="8766756"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>54536</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B90C982C-4D23-3371-8B11-3229F28C6FC7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="203200"/>
+          <a:ext cx="7772400" cy="4931336"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>199524</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{473D6F87-511D-DF15-D231-427548454E1B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="5283200"/>
+          <a:ext cx="7772400" cy="5279524"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>159290</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4D0C58FC-E98F-B295-A074-5E6034D4B110}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="203200"/>
+          <a:ext cx="7772400" cy="8287290"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>793750</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>311150</xdr:colOff>
+      <xdr:row>55</xdr:row>
+      <xdr:rowOff>12700</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E6C98619-9986-1031-CD71-42035D8FD1E7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="793750" y="8483600"/>
+          <a:ext cx="7772400" cy="2705100"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>67</xdr:row>
+      <xdr:rowOff>153123</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D0B6CCC5-3E4F-9FF4-342D-7A7019D06490}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="11582400"/>
+          <a:ext cx="7772400" cy="2185123"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>69</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>342900</xdr:colOff>
+      <xdr:row>84</xdr:row>
+      <xdr:rowOff>121239</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Picture 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6464CFFC-A822-46CB-F913-B29AB40A55EA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="825500" y="14020800"/>
+          <a:ext cx="7772400" cy="3169239"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -410,6 +1004,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -419,5 +1014,26 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69133511-A7DA-3247-A4F7-E84D013CD224}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E6EA2D9-4A8B-5A4B-B68A-E93771950F82}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>